<commit_message>
agregado link al drive videos scrum
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyeto/Evidencias de documentación/Burndown_RutaGest sprint 2.xlsx
+++ b/Fase 2/Evidencias Proyeto/Evidencias de documentación/Burndown_RutaGest sprint 2.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="spWRFUiLHLwZY+zRTzYEXkbYKR8QcL7ndlr9RPbJZyo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="POfOwWKGGs3fk64xVXjHHypwMQ8LmZU1eeSqqHpw7ws="/>
     </ext>
   </extLst>
 </workbook>
@@ -49,12 +49,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -102,20 +108,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -134,19 +135,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="1" i="0" sz="1800">
+              <a:defRPr b="1" i="0" sz="2000">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="757575"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="1" i="0" sz="1800">
+              <a:rPr b="1" i="0" sz="2000">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="757575"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
+                <a:latin typeface="+mn-lt"/>
               </a:rPr>
               <a:t>Burndown Chart – RutaGest (Semanas 6-8)</a:t>
             </a:r>
@@ -165,16 +166,25 @@
             <c:v>SP Ideal (planificado)</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:ln cmpd="sng" w="28575">
               <a:solidFill>
-                <a:srgbClr val="4A7EBB">
-                  <a:alpha val="100000"/>
-                </a:srgbClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
           </c:marker>
           <c:cat>
             <c:strRef>
@@ -187,7 +197,7 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -196,16 +206,25 @@
             <c:v>SP Real (avance actual)</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:ln cmpd="sng" w="28575">
               <a:solidFill>
-                <a:srgbClr val="BE4B48">
-                  <a:alpha val="100000"/>
-                </a:srgbClr>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
           </c:marker>
           <c:cat>
             <c:strRef>
@@ -218,13 +237,13 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="695300035"/>
-        <c:axId val="983710089"/>
+        <c:axId val="2045080379"/>
+        <c:axId val="7810206"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="695300035"/>
+        <c:axId val="2045080379"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -237,21 +256,21 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr lvl="0">
-                  <a:defRPr b="1" i="0" sz="1000">
+                  <a:defRPr b="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="Calibri"/>
+                    <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="1" i="0" sz="1000">
+                  <a:rPr b="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="Calibri"/>
+                    <a:latin typeface="+mn-lt"/>
                   </a:rPr>
-                  <a:t>Semana</a:t>
+                  <a:t/>
                 </a:r>
               </a:p>
             </c:rich>
@@ -271,22 +290,21 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0" i="0" sz="1000">
+              <a:defRPr b="0" i="0" sz="900">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="983710089"/>
+        <c:crossAx val="7810206"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="983710089"/>
+        <c:axId val="7810206"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="0.0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -306,21 +324,21 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr lvl="0">
-                  <a:defRPr b="1" i="0" sz="1000">
+                  <a:defRPr b="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="Calibri"/>
+                    <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="1" i="0" sz="1000">
+                  <a:rPr b="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="Calibri"/>
+                    <a:latin typeface="+mn-lt"/>
                   </a:rPr>
-                  <a:t>Story Points restantes</a:t>
+                  <a:t/>
                 </a:r>
               </a:p>
             </c:rich>
@@ -341,31 +359,31 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0" i="0" sz="1000">
+              <a:defRPr b="0" i="0" sz="900">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="695300035"/>
+        <c:crossAx val="2045080379"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
         <a:p>
           <a:pPr lvl="0">
-            <a:defRPr b="0" i="0" sz="1000">
+            <a:defRPr b="0" i="0" sz="900">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="1A1A1A"/>
               </a:solidFill>
-              <a:latin typeface="Calibri"/>
+              <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -373,11 +391,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-  </c:spPr>
 </c:chartSpace>
 </file>
 
@@ -386,14 +399,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6858000" cy="4133850"/>
+    <xdr:ext cx="9010650" cy="5486400"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1443044555" name="Chart 1" title="Gráfico"/>
+        <xdr:cNvPr id="526632875" name="Chart 1" title="Gráfico"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -622,76 +635,76 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>41.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>41.0</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6">
-        <f t="shared" ref="B3:C3" si="1">41-3</f>
+      <c r="B3" s="4">
+        <f>41-3</f>
         <v>38</v>
       </c>
-      <c r="C3" s="6">
-        <f t="shared" si="1"/>
-        <v>38</v>
-      </c>
-      <c r="E3" s="4"/>
+      <c r="C3" s="4">
+        <f>41</f>
+        <v>41</v>
+      </c>
+      <c r="E3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <f>B3-19</f>
         <v>19</v>
       </c>
-      <c r="C4" s="6">
-        <f>C3-27</f>
-        <v>11</v>
-      </c>
-      <c r="E4" s="4"/>
+      <c r="C4" s="4">
+        <f>41-3</f>
+        <v>38</v>
+      </c>
+      <c r="E4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <f>B4-15</f>
         <v>4</v>
       </c>
-      <c r="C5" s="6">
-        <f>C4-8</f>
-        <v>3</v>
+      <c r="C5" s="4">
+        <f>C4-27</f>
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <f>B5-4</f>
         <v>0</v>
       </c>
-      <c r="C6" s="6">
-        <f>C5-3</f>
+      <c r="C6" s="4">
+        <f>C5-11</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>